<commit_message>
Fix ALLO conditional rule values
</commit_message>
<xml_diff>
--- a/Преобразование Разделов.xlsx
+++ b/Преобразование Разделов.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Kezhunya/Documents/New project/MAUDAU/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Kezhunya/Documents/New project/АЛЛО/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{437B7FE7-EEB6-1248-BEC6-EC2ADE9578F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{430B7EA0-5183-3543-9C85-CDEA6E5F243E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16100" firstSheet="10" activeTab="18" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16100" firstSheet="16" activeTab="23" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Смесители" sheetId="1" r:id="rId1"/>
@@ -145,7 +145,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2990" uniqueCount="1873">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2992" uniqueCount="1874">
   <si>
     <t>№</t>
   </si>
@@ -5795,6 +5795,9 @@
   </si>
   <si>
     <t>Добавить параметры и подтянуть значения к канонам из описаний. Подсмотреть некоторые примеры как формирует генератор АЛЛО</t>
+  </si>
+  <si>
+    <t>Смыв=tornado</t>
   </si>
 </sst>
 </file>
@@ -6248,7 +6251,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10"/>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -6416,6 +6419,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="14" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -6438,14 +6453,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="14" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="13" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -6828,7 +6844,7 @@
       </c>
     </row>
     <row r="5" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="57">
+      <c r="A5" s="61">
         <v>2</v>
       </c>
       <c r="B5" s="15" t="s">
@@ -6844,7 +6860,7 @@
       </c>
     </row>
     <row r="6" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="58"/>
+      <c r="A6" s="62"/>
       <c r="B6" s="15" t="s">
         <v>13</v>
       </c>
@@ -6890,7 +6906,7 @@
       </c>
     </row>
     <row r="9" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="57">
+      <c r="A9" s="61">
         <v>5</v>
       </c>
       <c r="B9" s="15" t="s">
@@ -6906,7 +6922,7 @@
       </c>
     </row>
     <row r="10" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="58"/>
+      <c r="A10" s="62"/>
       <c r="B10" s="15" t="s">
         <v>24</v>
       </c>
@@ -8300,7 +8316,7 @@
       <c r="F29" s="53" t="s">
         <v>705</v>
       </c>
-      <c r="G29" s="64" t="s">
+      <c r="G29" s="68" t="s">
         <v>1868</v>
       </c>
     </row>
@@ -8320,7 +8336,7 @@
       <c r="F30" s="53" t="s">
         <v>705</v>
       </c>
-      <c r="G30" s="65"/>
+      <c r="G30" s="69"/>
     </row>
     <row r="31" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="15">
@@ -8338,7 +8354,7 @@
       <c r="F31" s="53" t="s">
         <v>705</v>
       </c>
-      <c r="G31" s="65"/>
+      <c r="G31" s="69"/>
     </row>
     <row r="32" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="15">
@@ -8356,7 +8372,7 @@
       <c r="F32" s="53" t="s">
         <v>705</v>
       </c>
-      <c r="G32" s="65"/>
+      <c r="G32" s="69"/>
     </row>
     <row r="33" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="15">
@@ -8374,7 +8390,7 @@
       <c r="F33" s="53" t="s">
         <v>705</v>
       </c>
-      <c r="G33" s="65"/>
+      <c r="G33" s="69"/>
     </row>
     <row r="34" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="15">
@@ -8392,7 +8408,7 @@
       <c r="F34" s="53" t="s">
         <v>705</v>
       </c>
-      <c r="G34" s="65"/>
+      <c r="G34" s="69"/>
     </row>
     <row r="35" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="15">
@@ -8410,7 +8426,7 @@
       <c r="F35" s="53" t="s">
         <v>705</v>
       </c>
-      <c r="G35" s="65"/>
+      <c r="G35" s="69"/>
     </row>
     <row r="36" spans="1:7" ht="10" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A36" s="6"/>
@@ -8419,7 +8435,7 @@
       <c r="D36" s="6"/>
       <c r="E36" s="6"/>
       <c r="F36" s="54"/>
-      <c r="G36" s="65"/>
+      <c r="G36" s="69"/>
     </row>
     <row r="37" spans="1:7" ht="22" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A37" s="4"/>
@@ -8434,7 +8450,7 @@
       <c r="F37" s="55" t="s">
         <v>6</v>
       </c>
-      <c r="G37" s="65"/>
+      <c r="G37" s="69"/>
     </row>
     <row r="38" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="15">
@@ -8451,7 +8467,7 @@
       <c r="F38" s="53" t="s">
         <v>713</v>
       </c>
-      <c r="G38" s="65"/>
+      <c r="G38" s="69"/>
     </row>
     <row r="39" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="15">
@@ -8469,7 +8485,7 @@
       <c r="F39" s="53" t="s">
         <v>713</v>
       </c>
-      <c r="G39" s="65"/>
+      <c r="G39" s="69"/>
     </row>
     <row r="40" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="15">
@@ -8487,7 +8503,7 @@
       <c r="F40" s="53" t="s">
         <v>713</v>
       </c>
-      <c r="G40" s="65"/>
+      <c r="G40" s="69"/>
     </row>
     <row r="41" spans="1:7" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A41" s="15">
@@ -8505,7 +8521,7 @@
       <c r="F41" s="53" t="s">
         <v>713</v>
       </c>
-      <c r="G41" s="66"/>
+      <c r="G41" s="70"/>
     </row>
     <row r="42" spans="1:7" ht="10" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A42" s="6"/>
@@ -14758,10 +14774,10 @@
       <c r="C4" s="44"/>
       <c r="D4" s="45"/>
       <c r="E4" s="44"/>
-      <c r="F4" s="67" t="s">
+      <c r="F4" s="57" t="s">
         <v>1099</v>
       </c>
-      <c r="G4" s="64" t="s">
+      <c r="G4" s="68" t="s">
         <v>1872</v>
       </c>
     </row>
@@ -14775,10 +14791,10 @@
       <c r="C5" s="44"/>
       <c r="D5" s="45"/>
       <c r="E5" s="44"/>
-      <c r="F5" s="67" t="s">
+      <c r="F5" s="57" t="s">
         <v>1101</v>
       </c>
-      <c r="G5" s="65"/>
+      <c r="G5" s="69"/>
     </row>
     <row r="6" spans="1:7" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="44">
@@ -14790,10 +14806,10 @@
       <c r="C6" s="44"/>
       <c r="D6" s="45"/>
       <c r="E6" s="44"/>
-      <c r="F6" s="67" t="s">
+      <c r="F6" s="57" t="s">
         <v>1103</v>
       </c>
-      <c r="G6" s="65"/>
+      <c r="G6" s="69"/>
     </row>
     <row r="7" spans="1:7" ht="32" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="44">
@@ -14805,10 +14821,10 @@
       <c r="C7" s="44"/>
       <c r="D7" s="45"/>
       <c r="E7" s="44"/>
-      <c r="F7" s="67" t="s">
+      <c r="F7" s="57" t="s">
         <v>1105</v>
       </c>
-      <c r="G7" s="65"/>
+      <c r="G7" s="69"/>
     </row>
     <row r="8" spans="1:7" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A8" s="42"/>
@@ -14820,10 +14836,10 @@
         <v>5</v>
       </c>
       <c r="E8" s="42"/>
-      <c r="F8" s="68" t="s">
+      <c r="F8" s="58" t="s">
         <v>6</v>
       </c>
-      <c r="G8" s="65"/>
+      <c r="G8" s="69"/>
     </row>
     <row r="9" spans="1:7" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="44">
@@ -14835,10 +14851,10 @@
       <c r="C9" s="44"/>
       <c r="D9" s="45"/>
       <c r="E9" s="44"/>
-      <c r="F9" s="67" t="s">
+      <c r="F9" s="57" t="s">
         <v>1870</v>
       </c>
-      <c r="G9" s="65"/>
+      <c r="G9" s="69"/>
     </row>
     <row r="10" spans="1:7" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="44">
@@ -14850,10 +14866,10 @@
       <c r="C10" s="44"/>
       <c r="D10" s="45"/>
       <c r="E10" s="44"/>
-      <c r="F10" s="67" t="s">
+      <c r="F10" s="57" t="s">
         <v>1109</v>
       </c>
-      <c r="G10" s="65"/>
+      <c r="G10" s="69"/>
     </row>
     <row r="11" spans="1:7" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="44">
@@ -14865,10 +14881,10 @@
       <c r="C11" s="44"/>
       <c r="D11" s="45"/>
       <c r="E11" s="44"/>
-      <c r="F11" s="67" t="s">
+      <c r="F11" s="57" t="s">
         <v>1111</v>
       </c>
-      <c r="G11" s="65"/>
+      <c r="G11" s="69"/>
     </row>
     <row r="12" spans="1:7" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="44">
@@ -14880,10 +14896,10 @@
       <c r="C12" s="44"/>
       <c r="D12" s="45"/>
       <c r="E12" s="44"/>
-      <c r="F12" s="67" t="s">
+      <c r="F12" s="57" t="s">
         <v>1113</v>
       </c>
-      <c r="G12" s="65"/>
+      <c r="G12" s="69"/>
     </row>
     <row r="13" spans="1:7" ht="32" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A13" s="44">
@@ -14895,10 +14911,10 @@
       <c r="C13" s="44"/>
       <c r="D13" s="45"/>
       <c r="E13" s="44"/>
-      <c r="F13" s="67" t="s">
+      <c r="F13" s="57" t="s">
         <v>1115</v>
       </c>
-      <c r="G13" s="65"/>
+      <c r="G13" s="69"/>
     </row>
     <row r="14" spans="1:7" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A14" s="42"/>
@@ -14910,10 +14926,10 @@
         <v>5</v>
       </c>
       <c r="E14" s="42"/>
-      <c r="F14" s="68" t="s">
+      <c r="F14" s="58" t="s">
         <v>6</v>
       </c>
-      <c r="G14" s="65"/>
+      <c r="G14" s="69"/>
     </row>
     <row r="15" spans="1:7" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="44">
@@ -14925,10 +14941,10 @@
       <c r="C15" s="44"/>
       <c r="D15" s="45"/>
       <c r="E15" s="44"/>
-      <c r="F15" s="67" t="s">
+      <c r="F15" s="57" t="s">
         <v>1118</v>
       </c>
-      <c r="G15" s="65"/>
+      <c r="G15" s="69"/>
     </row>
     <row r="16" spans="1:7" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="44">
@@ -14940,10 +14956,10 @@
       <c r="C16" s="44"/>
       <c r="D16" s="45"/>
       <c r="E16" s="44"/>
-      <c r="F16" s="69" t="s">
+      <c r="F16" s="59" t="s">
         <v>1120</v>
       </c>
-      <c r="G16" s="65"/>
+      <c r="G16" s="69"/>
     </row>
     <row r="17" spans="1:7" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="44">
@@ -14955,10 +14971,10 @@
       <c r="C17" s="44"/>
       <c r="D17" s="45"/>
       <c r="E17" s="44"/>
-      <c r="F17" s="67" t="s">
+      <c r="F17" s="57" t="s">
         <v>1122</v>
       </c>
-      <c r="G17" s="65"/>
+      <c r="G17" s="69"/>
     </row>
     <row r="18" spans="1:7" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="44">
@@ -14970,10 +14986,10 @@
       <c r="C18" s="44"/>
       <c r="D18" s="45"/>
       <c r="E18" s="44"/>
-      <c r="F18" s="69" t="s">
+      <c r="F18" s="59" t="s">
         <v>1124</v>
       </c>
-      <c r="G18" s="65"/>
+      <c r="G18" s="69"/>
     </row>
     <row r="19" spans="1:7" ht="32" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A19" s="44">
@@ -14985,10 +15001,10 @@
       <c r="C19" s="44"/>
       <c r="D19" s="45"/>
       <c r="E19" s="44"/>
-      <c r="F19" s="67" t="s">
+      <c r="F19" s="57" t="s">
         <v>1126</v>
       </c>
-      <c r="G19" s="65"/>
+      <c r="G19" s="69"/>
     </row>
     <row r="20" spans="1:7" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A20" s="42"/>
@@ -15000,10 +15016,10 @@
         <v>5</v>
       </c>
       <c r="E20" s="42"/>
-      <c r="F20" s="68" t="s">
+      <c r="F20" s="58" t="s">
         <v>6</v>
       </c>
-      <c r="G20" s="65"/>
+      <c r="G20" s="69"/>
     </row>
     <row r="21" spans="1:7" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="44">
@@ -15015,10 +15031,10 @@
       <c r="C21" s="44"/>
       <c r="D21" s="45"/>
       <c r="E21" s="44"/>
-      <c r="F21" s="69" t="s">
+      <c r="F21" s="59" t="s">
         <v>1129</v>
       </c>
-      <c r="G21" s="65"/>
+      <c r="G21" s="69"/>
     </row>
     <row r="22" spans="1:7" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="44">
@@ -15030,10 +15046,10 @@
       <c r="C22" s="44"/>
       <c r="D22" s="45"/>
       <c r="E22" s="44"/>
-      <c r="F22" s="69" t="s">
+      <c r="F22" s="59" t="s">
         <v>1131</v>
       </c>
-      <c r="G22" s="65"/>
+      <c r="G22" s="69"/>
     </row>
     <row r="23" spans="1:7" ht="32" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A23" s="44">
@@ -15045,10 +15061,10 @@
       <c r="C23" s="44"/>
       <c r="D23" s="45"/>
       <c r="E23" s="44"/>
-      <c r="F23" s="67" t="s">
+      <c r="F23" s="57" t="s">
         <v>1133</v>
       </c>
-      <c r="G23" s="66"/>
+      <c r="G23" s="70"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" s="47"/>
@@ -16856,7 +16872,7 @@
 
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1700-000000000000}">
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
@@ -16909,15 +16925,15 @@
       <c r="A4" s="24">
         <v>1</v>
       </c>
-      <c r="B4" s="25" t="s">
+      <c r="B4" s="10" t="s">
         <v>1215</v>
       </c>
       <c r="C4" s="10"/>
-      <c r="D4" s="25" t="s">
+      <c r="D4" s="10" t="s">
         <v>1216</v>
       </c>
       <c r="E4" s="10"/>
-      <c r="F4" s="26" t="s">
+      <c r="F4" s="60" t="s">
         <v>1217</v>
       </c>
     </row>
@@ -17063,254 +17079,269 @@
         <v>6</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="24">
+    <row r="15" spans="1:6" s="73" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="74">
         <v>10</v>
       </c>
-      <c r="B15" s="25" t="s">
-        <v>1235</v>
-      </c>
-      <c r="C15" s="10"/>
-      <c r="D15" s="10"/>
-      <c r="E15" s="10"/>
+      <c r="B15" s="10" t="s">
+        <v>1873</v>
+      </c>
+      <c r="C15" s="71"/>
+      <c r="D15" s="72"/>
+      <c r="E15" s="71"/>
       <c r="F15" s="26" t="s">
         <v>1236</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="24">
+        <f>A15+1</f>
         <v>11</v>
       </c>
       <c r="B16" s="25" t="s">
-        <v>1237</v>
+        <v>1235</v>
       </c>
       <c r="C16" s="10"/>
       <c r="D16" s="10"/>
       <c r="E16" s="10"/>
-      <c r="F16" s="25" t="s">
-        <v>1238</v>
+      <c r="F16" s="26" t="s">
+        <v>1236</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="24">
+        <f t="shared" ref="A17:A30" si="0">A16+1</f>
         <v>12</v>
       </c>
       <c r="B17" s="25" t="s">
-        <v>1239</v>
+        <v>1237</v>
       </c>
       <c r="C17" s="10"/>
       <c r="D17" s="10"/>
       <c r="E17" s="10"/>
-      <c r="F17" s="26" t="s">
-        <v>1240</v>
+      <c r="F17" s="25" t="s">
+        <v>1238</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="24">
+        <f t="shared" si="0"/>
         <v>13</v>
       </c>
       <c r="B18" s="25" t="s">
-        <v>1241</v>
+        <v>1239</v>
       </c>
       <c r="C18" s="10"/>
       <c r="D18" s="10"/>
       <c r="E18" s="10"/>
       <c r="F18" s="26" t="s">
-        <v>1242</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+        <v>1240</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="24">
+        <f t="shared" si="0"/>
         <v>14</v>
       </c>
       <c r="B19" s="25" t="s">
-        <v>1243</v>
+        <v>1241</v>
       </c>
       <c r="C19" s="10"/>
       <c r="D19" s="10"/>
       <c r="E19" s="10"/>
-      <c r="F19" s="25" t="s">
-        <v>1244</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F19" s="26" t="s">
+        <v>1242</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="24">
+        <f t="shared" si="0"/>
         <v>15</v>
       </c>
       <c r="B20" s="25" t="s">
-        <v>1245</v>
+        <v>1243</v>
       </c>
       <c r="C20" s="10"/>
       <c r="D20" s="10"/>
       <c r="E20" s="10"/>
-      <c r="F20" s="26" t="s">
-        <v>1246</v>
+      <c r="F20" s="25" t="s">
+        <v>1244</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="24">
+        <f t="shared" si="0"/>
         <v>16</v>
       </c>
       <c r="B21" s="25" t="s">
-        <v>1247</v>
+        <v>1245</v>
       </c>
       <c r="C21" s="10"/>
       <c r="D21" s="10"/>
       <c r="E21" s="10"/>
       <c r="F21" s="26" t="s">
-        <v>1248</v>
+        <v>1246</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="24">
+        <f t="shared" si="0"/>
         <v>17</v>
       </c>
       <c r="B22" s="25" t="s">
-        <v>1249</v>
+        <v>1247</v>
       </c>
       <c r="C22" s="10"/>
       <c r="D22" s="10"/>
       <c r="E22" s="10"/>
       <c r="F22" s="26" t="s">
-        <v>1250</v>
+        <v>1248</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="24">
+        <f t="shared" si="0"/>
         <v>18</v>
       </c>
       <c r="B23" s="25" t="s">
-        <v>1251</v>
+        <v>1249</v>
       </c>
       <c r="C23" s="10"/>
       <c r="D23" s="10"/>
       <c r="E23" s="10"/>
-      <c r="F23" s="25" t="s">
-        <v>1252</v>
+      <c r="F23" s="26" t="s">
+        <v>1250</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="24">
+        <f t="shared" si="0"/>
         <v>19</v>
       </c>
       <c r="B24" s="25" t="s">
-        <v>1253</v>
+        <v>1251</v>
       </c>
       <c r="C24" s="10"/>
       <c r="D24" s="10"/>
       <c r="E24" s="10"/>
-      <c r="F24" s="26" t="s">
-        <v>1254</v>
+      <c r="F24" s="25" t="s">
+        <v>1252</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="24">
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="B25" s="25" t="s">
-        <v>1255</v>
+        <v>1253</v>
       </c>
       <c r="C25" s="10"/>
       <c r="D25" s="10"/>
       <c r="E25" s="10"/>
       <c r="F25" s="26" t="s">
-        <v>1256</v>
+        <v>1254</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="24">
+        <f t="shared" si="0"/>
         <v>21</v>
       </c>
       <c r="B26" s="25" t="s">
-        <v>1257</v>
+        <v>1255</v>
       </c>
       <c r="C26" s="10"/>
-      <c r="D26" s="25" t="s">
-        <v>1258</v>
-      </c>
+      <c r="D26" s="10"/>
       <c r="E26" s="10"/>
       <c r="F26" s="26" t="s">
-        <v>1259</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="24">
+        <f t="shared" si="0"/>
         <v>22</v>
       </c>
-      <c r="B27" s="25" t="s">
-        <v>1260</v>
+      <c r="B27" s="10" t="s">
+        <v>1257</v>
       </c>
       <c r="C27" s="10"/>
       <c r="D27" s="25" t="s">
-        <v>1261</v>
+        <v>1258</v>
       </c>
       <c r="E27" s="10"/>
       <c r="F27" s="26" t="s">
-        <v>1262</v>
+        <v>1259</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="24">
+        <f t="shared" si="0"/>
         <v>23</v>
       </c>
       <c r="B28" s="25" t="s">
-        <v>1263</v>
+        <v>1260</v>
       </c>
       <c r="C28" s="10"/>
-      <c r="D28" s="10"/>
+      <c r="D28" s="25" t="s">
+        <v>1261</v>
+      </c>
       <c r="E28" s="10"/>
       <c r="F28" s="26" t="s">
-        <v>1264</v>
+        <v>1262</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="24">
+        <f t="shared" si="0"/>
         <v>24</v>
       </c>
       <c r="B29" s="25" t="s">
-        <v>1265</v>
+        <v>1263</v>
       </c>
       <c r="C29" s="10"/>
       <c r="D29" s="10"/>
       <c r="E29" s="10"/>
       <c r="F29" s="26" t="s">
+        <v>1264</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="24">
+        <f t="shared" si="0"/>
+        <v>25</v>
+      </c>
+      <c r="B30" s="25" t="s">
+        <v>1265</v>
+      </c>
+      <c r="C30" s="10"/>
+      <c r="D30" s="10"/>
+      <c r="E30" s="10"/>
+      <c r="F30" s="26" t="s">
         <v>1266</v>
       </c>
     </row>
-    <row r="30" spans="1:6" ht="9" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="9"/>
-      <c r="B30" s="9"/>
-      <c r="C30" s="9"/>
-      <c r="D30" s="9"/>
-      <c r="E30" s="9"/>
-      <c r="F30" s="9"/>
-    </row>
-    <row r="31" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="8"/>
-      <c r="B31" s="22" t="s">
+    <row r="31" spans="1:6" ht="9" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="9"/>
+      <c r="B31" s="9"/>
+      <c r="C31" s="9"/>
+      <c r="D31" s="9"/>
+      <c r="E31" s="9"/>
+      <c r="F31" s="9"/>
+    </row>
+    <row r="32" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="8"/>
+      <c r="B32" s="22" t="s">
         <v>1267</v>
       </c>
-      <c r="C31" s="8"/>
-      <c r="D31" s="22" t="s">
+      <c r="C32" s="8"/>
+      <c r="D32" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="E31" s="8"/>
-      <c r="F31" s="23" t="s">
+      <c r="E32" s="8"/>
+      <c r="F32" s="23" t="s">
         <v>6</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="24">
-        <v>25</v>
-      </c>
-      <c r="B32" s="25" t="s">
-        <v>1268</v>
-      </c>
-      <c r="C32" s="10"/>
-      <c r="D32" s="10"/>
-      <c r="E32" s="10"/>
-      <c r="F32" s="26" t="s">
-        <v>1269</v>
       </c>
     </row>
     <row r="33" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -17318,92 +17349,112 @@
         <v>26</v>
       </c>
       <c r="B33" s="25" t="s">
-        <v>1270</v>
+        <v>1268</v>
       </c>
       <c r="C33" s="10"/>
       <c r="D33" s="10"/>
       <c r="E33" s="10"/>
       <c r="F33" s="26" t="s">
-        <v>1271</v>
+        <v>1269</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="24">
+        <f t="shared" ref="A33:A39" si="1">A33+1</f>
         <v>27</v>
       </c>
       <c r="B34" s="25" t="s">
-        <v>1272</v>
+        <v>1270</v>
       </c>
       <c r="C34" s="10"/>
       <c r="D34" s="10"/>
       <c r="E34" s="10"/>
-      <c r="F34" s="25" t="s">
-        <v>1273</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F34" s="26" t="s">
+        <v>1271</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="24">
+        <f t="shared" si="1"/>
         <v>28</v>
       </c>
       <c r="B35" s="25" t="s">
-        <v>1274</v>
+        <v>1272</v>
       </c>
       <c r="C35" s="10"/>
       <c r="D35" s="10"/>
       <c r="E35" s="10"/>
       <c r="F35" s="25" t="s">
-        <v>1275</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+        <v>1273</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="24">
+        <f t="shared" si="1"/>
         <v>29</v>
       </c>
       <c r="B36" s="25" t="s">
-        <v>1263</v>
+        <v>1274</v>
       </c>
       <c r="C36" s="10"/>
       <c r="D36" s="10"/>
       <c r="E36" s="10"/>
-      <c r="F36" s="26" t="s">
-        <v>1276</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F36" s="25" t="s">
+        <v>1275</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="24">
+        <f t="shared" si="1"/>
         <v>30</v>
       </c>
       <c r="B37" s="25" t="s">
-        <v>1277</v>
+        <v>1263</v>
       </c>
       <c r="C37" s="10"/>
       <c r="D37" s="10"/>
       <c r="E37" s="10"/>
       <c r="F37" s="26" t="s">
-        <v>1278</v>
+        <v>1276</v>
       </c>
     </row>
     <row r="38" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="24">
+        <f t="shared" si="1"/>
         <v>31</v>
       </c>
       <c r="B38" s="25" t="s">
-        <v>1279</v>
+        <v>1277</v>
       </c>
       <c r="C38" s="10"/>
       <c r="D38" s="10"/>
       <c r="E38" s="10"/>
       <c r="F38" s="26" t="s">
+        <v>1278</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="24">
+        <f t="shared" si="1"/>
+        <v>32</v>
+      </c>
+      <c r="B39" s="25" t="s">
+        <v>1279</v>
+      </c>
+      <c r="C39" s="10"/>
+      <c r="D39" s="10"/>
+      <c r="E39" s="10"/>
+      <c r="F39" s="26" t="s">
         <v>1280</v>
       </c>
     </row>
-    <row r="39" spans="1:6" ht="9" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="9"/>
-      <c r="B39" s="9"/>
-      <c r="C39" s="9"/>
-      <c r="D39" s="9"/>
-      <c r="E39" s="9"/>
-      <c r="F39" s="9"/>
+    <row r="40" spans="1:6" ht="9" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="9"/>
+      <c r="B40" s="9"/>
+      <c r="C40" s="9"/>
+      <c r="D40" s="9"/>
+      <c r="E40" s="9"/>
+      <c r="F40" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -23172,11 +23223,11 @@
     </row>
     <row r="30" spans="1:6" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A30" s="5"/>
-      <c r="B30" s="57" t="s">
+      <c r="B30" s="61" t="s">
         <v>351</v>
       </c>
-      <c r="C30" s="59"/>
-      <c r="D30" s="60"/>
+      <c r="C30" s="63"/>
+      <c r="D30" s="64"/>
       <c r="E30" s="5"/>
       <c r="F30" s="16" t="s">
         <v>352</v>
@@ -23242,10 +23293,10 @@
       </c>
     </row>
     <row r="4" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="61">
+      <c r="A4" s="65">
         <v>1</v>
       </c>
-      <c r="B4" s="63" t="s">
+      <c r="B4" s="67" t="s">
         <v>354</v>
       </c>
       <c r="C4" s="4"/>
@@ -23258,8 +23309,8 @@
       </c>
     </row>
     <row r="5" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="62"/>
-      <c r="B5" s="62"/>
+      <c r="A5" s="66"/>
+      <c r="B5" s="66"/>
       <c r="C5" s="4"/>
       <c r="D5" s="18" t="s">
         <v>216</v>

</xml_diff>